<commit_message>
feat: complete coordinator student tracking, dynamic drive process, and profile management
</commit_message>
<xml_diff>
--- a/bulk_upload_module/templates/sample_company_drives.xlsx
+++ b/bulk_upload_module/templates/sample_company_drives.xlsx
@@ -789,6 +789,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Product,Service,Consulting,Startup"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Active,Upcoming,Completed,Archived"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>